<commit_message>
Guerra de Mafias 3: Excel actualizado
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/guerra_mafias_3.xlsx
+++ b/data/guerra_mafias_3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\power bi\webhook\Produccion\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3998FB2-7332-4974-BC11-7DACEF006EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{871827B2-E8C9-49C9-9D2E-A933659ED72D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batallas" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1355" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1355" uniqueCount="203">
   <si>
     <t>player1</t>
   </si>
@@ -293,9 +293,6 @@
     <t>https://replay.pokemonshowdown.com/gen9randombattle-2701946499-8gpac1h4y6qgbcxyyx1t1dampiii9a6pw</t>
   </si>
   <si>
-    <t>Josar</t>
-  </si>
-  <si>
     <t>https://replay.pokemonshowdown.com/gen8vgc2021-2701703506</t>
   </si>
   <si>
@@ -311,18 +308,12 @@
     <t>https://replay.pokemonshowdown.com/gen9monotyperandombattle-2701685590</t>
   </si>
   <si>
-    <t>Arnaenaed ∾</t>
-  </si>
-  <si>
     <t>https://replay.pokemonshowdown.com/gen8vgc2021-2700127756</t>
   </si>
   <si>
     <t>https://replay.pokemonshowdown.com/gen9nationaldexmonotype-2697860912</t>
   </si>
   <si>
-    <t>zeedra</t>
-  </si>
-  <si>
     <t>https://replay.pokemonshowdown.com/gen9nationaldexmonotype-2700276310</t>
   </si>
   <si>
@@ -456,9 +447,6 @@
   </si>
   <si>
     <t>Willy</t>
-  </si>
-  <si>
-    <t>Mouka</t>
   </si>
   <si>
     <t>https://replay.pokemonshowdown.com/gen9randombattle-2696332664</t>
@@ -1133,13 +1121,13 @@
         <v>31</v>
       </c>
       <c r="H2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I2" t="s">
         <v>32</v>
       </c>
       <c r="J2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="L2" t="s">
         <v>33</v>
@@ -1174,10 +1162,10 @@
         <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D3" t="s">
         <v>28</v>
@@ -1192,13 +1180,13 @@
         <v>31</v>
       </c>
       <c r="H3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I3" t="s">
         <v>32</v>
       </c>
       <c r="J3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="L3" t="s">
         <v>33</v>
@@ -1251,13 +1239,13 @@
         <v>31</v>
       </c>
       <c r="H4" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="I4" t="s">
         <v>32</v>
       </c>
       <c r="J4" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="L4" t="s">
         <v>33</v>
@@ -1310,13 +1298,13 @@
         <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I5" t="s">
         <v>32</v>
       </c>
       <c r="J5" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L5" t="s">
         <v>43</v>
@@ -1369,13 +1357,13 @@
         <v>31</v>
       </c>
       <c r="H6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I6" t="s">
         <v>32</v>
       </c>
       <c r="J6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="L6" t="s">
         <v>43</v>
@@ -1428,13 +1416,13 @@
         <v>31</v>
       </c>
       <c r="H7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I7" t="s">
         <v>32</v>
       </c>
       <c r="J7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L7" t="s">
         <v>43</v>
@@ -1466,7 +1454,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B8" t="s">
         <v>26</v>
@@ -1487,13 +1475,13 @@
         <v>31</v>
       </c>
       <c r="H8" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="I8" t="s">
         <v>32</v>
       </c>
       <c r="J8" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="L8" t="s">
         <v>33</v>
@@ -1525,13 +1513,13 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B9" t="s">
         <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D9" t="s">
         <v>28</v>
@@ -1585,13 +1573,13 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B10" t="s">
         <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D10" t="s">
         <v>28</v>
@@ -1606,13 +1594,13 @@
         <v>31</v>
       </c>
       <c r="H10" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I10" t="s">
         <v>32</v>
       </c>
       <c r="J10" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="L10" t="s">
         <v>33</v>
@@ -1665,13 +1653,13 @@
         <v>31</v>
       </c>
       <c r="H11" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I11" t="s">
         <v>32</v>
       </c>
       <c r="J11" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L11" t="s">
         <v>43</v>
@@ -1724,13 +1712,13 @@
         <v>31</v>
       </c>
       <c r="H12" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I12" t="s">
         <v>32</v>
       </c>
       <c r="J12" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="L12" t="s">
         <v>43</v>
@@ -1783,13 +1771,13 @@
         <v>31</v>
       </c>
       <c r="H13" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I13" t="s">
         <v>32</v>
       </c>
       <c r="J13" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L13" t="s">
         <v>43</v>
@@ -1821,13 +1809,13 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B14" t="s">
         <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D14" t="s">
         <v>28</v>
@@ -1842,13 +1830,13 @@
         <v>31</v>
       </c>
       <c r="H14" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="I14" t="s">
         <v>32</v>
       </c>
       <c r="J14" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="L14" t="s">
         <v>50</v>
@@ -1880,13 +1868,13 @@
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B15" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C15" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D15" t="s">
         <v>28</v>
@@ -1901,13 +1889,13 @@
         <v>31</v>
       </c>
       <c r="H15" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="I15" t="s">
         <v>32</v>
       </c>
       <c r="J15" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="L15" t="s">
         <v>43</v>
@@ -1939,13 +1927,13 @@
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B16" t="s">
         <v>62</v>
       </c>
       <c r="C16" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D16" t="s">
         <v>28</v>
@@ -1960,13 +1948,13 @@
         <v>31</v>
       </c>
       <c r="H16" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="I16" t="s">
         <v>32</v>
       </c>
       <c r="J16" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="L16" t="s">
         <v>43</v>
@@ -2001,7 +1989,7 @@
         <v>58</v>
       </c>
       <c r="B17" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C17" t="s">
         <v>58</v>
@@ -2019,13 +2007,13 @@
         <v>31</v>
       </c>
       <c r="H17" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I17" t="s">
         <v>32</v>
       </c>
       <c r="J17" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L17" t="s">
         <v>43</v>
@@ -2060,10 +2048,10 @@
         <v>58</v>
       </c>
       <c r="B18" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C18" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D18" t="s">
         <v>28</v>
@@ -2078,13 +2066,13 @@
         <v>31</v>
       </c>
       <c r="H18" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I18" t="s">
         <v>32</v>
       </c>
       <c r="J18" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L18" t="s">
         <v>43</v>
@@ -2116,13 +2104,13 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B19" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C19" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
@@ -2137,13 +2125,13 @@
         <v>31</v>
       </c>
       <c r="H19" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="I19" t="s">
         <v>32</v>
       </c>
       <c r="J19" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="L19" t="s">
         <v>33</v>
@@ -2175,7 +2163,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B20" t="s">
         <v>58</v>
@@ -2196,13 +2184,13 @@
         <v>31</v>
       </c>
       <c r="H20" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="I20" t="s">
         <v>32</v>
       </c>
       <c r="J20" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="L20" t="s">
         <v>50</v>
@@ -2234,7 +2222,7 @@
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B21" t="s">
         <v>62</v>
@@ -2255,13 +2243,13 @@
         <v>31</v>
       </c>
       <c r="H21" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="I21" t="s">
         <v>32</v>
       </c>
       <c r="J21" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="L21" t="s">
         <v>33</v>
@@ -2296,10 +2284,10 @@
         <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C22" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D22" t="s">
         <v>28</v>
@@ -2314,13 +2302,13 @@
         <v>31</v>
       </c>
       <c r="H22" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I22" t="s">
         <v>32</v>
       </c>
       <c r="J22" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L22" t="s">
         <v>43</v>
@@ -2355,10 +2343,10 @@
         <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C23" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D23" t="s">
         <v>28</v>
@@ -2373,13 +2361,13 @@
         <v>31</v>
       </c>
       <c r="H23" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I23" t="s">
         <v>32</v>
       </c>
       <c r="J23" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="L23" t="s">
         <v>43</v>
@@ -2411,13 +2399,13 @@
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B24" t="s">
         <v>72</v>
       </c>
       <c r="C24" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D24" t="s">
         <v>28</v>
@@ -2432,13 +2420,13 @@
         <v>31</v>
       </c>
       <c r="H24" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I24" t="s">
         <v>32</v>
       </c>
       <c r="J24" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="L24" t="s">
         <v>43</v>
@@ -2473,7 +2461,7 @@
         <v>72</v>
       </c>
       <c r="B25" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C25" t="s">
         <v>72</v>
@@ -2491,13 +2479,13 @@
         <v>31</v>
       </c>
       <c r="H25" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I25" t="s">
         <v>32</v>
       </c>
       <c r="J25" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="L25" t="s">
         <v>43</v>
@@ -2550,13 +2538,13 @@
         <v>31</v>
       </c>
       <c r="H26" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I26" t="s">
         <v>32</v>
       </c>
       <c r="J26" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L26" t="s">
         <v>43</v>
@@ -2591,10 +2579,10 @@
         <v>72</v>
       </c>
       <c r="B27" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D27" t="s">
         <v>28</v>
@@ -2609,13 +2597,13 @@
         <v>31</v>
       </c>
       <c r="H27" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I27" t="s">
         <v>32</v>
       </c>
       <c r="J27" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="L27" t="s">
         <v>43</v>
@@ -2668,13 +2656,13 @@
         <v>31</v>
       </c>
       <c r="H28" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I28" t="s">
         <v>32</v>
       </c>
       <c r="J28" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="L28" t="s">
         <v>43</v>
@@ -2709,10 +2697,10 @@
         <v>77</v>
       </c>
       <c r="B29" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D29" t="s">
         <v>28</v>
@@ -2727,13 +2715,13 @@
         <v>31</v>
       </c>
       <c r="H29" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I29" t="s">
         <v>32</v>
       </c>
       <c r="J29" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L29" t="s">
         <v>43</v>
@@ -2765,13 +2753,13 @@
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B30" t="s">
         <v>72</v>
       </c>
       <c r="C30" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D30" t="s">
         <v>28</v>
@@ -2786,13 +2774,13 @@
         <v>31</v>
       </c>
       <c r="H30" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I30" t="s">
         <v>32</v>
       </c>
       <c r="J30" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L30" t="s">
         <v>43</v>
@@ -2824,13 +2812,13 @@
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B31" t="s">
         <v>77</v>
       </c>
       <c r="C31" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D31" t="s">
         <v>28</v>
@@ -2845,13 +2833,13 @@
         <v>31</v>
       </c>
       <c r="H31" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I31" t="s">
         <v>32</v>
       </c>
       <c r="J31" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L31" t="s">
         <v>43</v>
@@ -2883,13 +2871,13 @@
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B32" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C32" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D32" t="s">
         <v>28</v>
@@ -2904,13 +2892,13 @@
         <v>31</v>
       </c>
       <c r="H32" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I32" t="s">
         <v>32</v>
       </c>
       <c r="J32" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="L32" t="s">
         <v>50</v>
@@ -2928,7 +2916,7 @@
         <v>0</v>
       </c>
       <c r="S32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="T32">
         <v>8</v>
@@ -2937,18 +2925,18 @@
         <v>28</v>
       </c>
       <c r="AA32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>165</v>
+      </c>
+      <c r="B33" t="s">
         <v>169</v>
       </c>
-      <c r="B33" t="s">
-        <v>173</v>
-      </c>
       <c r="C33" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D33" t="s">
         <v>28</v>
@@ -2963,13 +2951,13 @@
         <v>31</v>
       </c>
       <c r="H33" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I33" t="s">
         <v>32</v>
       </c>
       <c r="J33" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="L33" t="s">
         <v>43</v>
@@ -2987,7 +2975,7 @@
         <v>0</v>
       </c>
       <c r="S33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="T33">
         <v>9</v>
@@ -2996,18 +2984,18 @@
         <v>28</v>
       </c>
       <c r="AA33" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B34" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C34" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D34" t="s">
         <v>28</v>
@@ -3022,13 +3010,13 @@
         <v>31</v>
       </c>
       <c r="H34" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I34" t="s">
         <v>32</v>
       </c>
       <c r="J34" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="L34" t="s">
         <v>43</v>
@@ -3046,7 +3034,7 @@
         <v>0</v>
       </c>
       <c r="S34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="T34">
         <v>9</v>
@@ -3055,15 +3043,15 @@
         <v>28</v>
       </c>
       <c r="AA34" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B35" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C35" t="s">
         <v>27</v>
@@ -3081,13 +3069,13 @@
         <v>31</v>
       </c>
       <c r="H35" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I35" t="s">
         <v>32</v>
       </c>
       <c r="J35" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="L35" t="s">
         <v>43</v>
@@ -3114,18 +3102,18 @@
         <v>28</v>
       </c>
       <c r="AA35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C36" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D36" t="s">
         <v>28</v>
@@ -3140,13 +3128,13 @@
         <v>31</v>
       </c>
       <c r="H36" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I36" t="s">
         <v>32</v>
       </c>
       <c r="J36" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="L36" t="s">
         <v>50</v>
@@ -3164,7 +3152,7 @@
         <v>0</v>
       </c>
       <c r="S36" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="T36">
         <v>8</v>
@@ -3173,18 +3161,18 @@
         <v>28</v>
       </c>
       <c r="AA36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B37" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D37" t="s">
         <v>28</v>
@@ -3199,13 +3187,13 @@
         <v>31</v>
       </c>
       <c r="H37" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I37" t="s">
         <v>32</v>
       </c>
       <c r="J37" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="L37" t="s">
         <v>43</v>
@@ -3223,7 +3211,7 @@
         <v>0</v>
       </c>
       <c r="S37" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="T37">
         <v>9</v>
@@ -3232,18 +3220,18 @@
         <v>28</v>
       </c>
       <c r="AA37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B38" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C38" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D38" t="s">
         <v>28</v>
@@ -3258,13 +3246,13 @@
         <v>31</v>
       </c>
       <c r="H38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I38" t="s">
         <v>32</v>
       </c>
       <c r="J38" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="L38" t="s">
         <v>50</v>
@@ -3282,7 +3270,7 @@
         <v>0</v>
       </c>
       <c r="S38" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="T38">
         <v>9</v>
@@ -3291,18 +3279,18 @@
         <v>28</v>
       </c>
       <c r="AA38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B39" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C39" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D39" t="s">
         <v>28</v>
@@ -3317,13 +3305,13 @@
         <v>31</v>
       </c>
       <c r="H39" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I39" t="s">
         <v>32</v>
       </c>
       <c r="J39" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="L39" t="s">
         <v>43</v>
@@ -3341,7 +3329,7 @@
         <v>0</v>
       </c>
       <c r="S39" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="T39">
         <v>9</v>
@@ -3350,18 +3338,18 @@
         <v>28</v>
       </c>
       <c r="AA39" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B40" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C40" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D40" t="s">
         <v>28</v>
@@ -3376,13 +3364,13 @@
         <v>31</v>
       </c>
       <c r="H40" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I40" t="s">
         <v>32</v>
       </c>
       <c r="J40" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L40" t="s">
         <v>43</v>
@@ -3400,7 +3388,7 @@
         <v>0</v>
       </c>
       <c r="S40" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="T40">
         <v>9</v>
@@ -3409,18 +3397,18 @@
         <v>28</v>
       </c>
       <c r="AA40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B41" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C41" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D41" t="s">
         <v>28</v>
@@ -3435,13 +3423,13 @@
         <v>31</v>
       </c>
       <c r="H41" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I41" t="s">
         <v>32</v>
       </c>
       <c r="J41" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L41" t="s">
         <v>43</v>
@@ -3459,7 +3447,7 @@
         <v>0</v>
       </c>
       <c r="S41" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="T41">
         <v>9</v>
@@ -3468,18 +3456,18 @@
         <v>28</v>
       </c>
       <c r="AA41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B42" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C42" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D42" t="s">
         <v>28</v>
@@ -3494,13 +3482,13 @@
         <v>31</v>
       </c>
       <c r="H42" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I42" t="s">
         <v>32</v>
       </c>
       <c r="J42" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="L42" t="s">
         <v>43</v>
@@ -3518,7 +3506,7 @@
         <v>0</v>
       </c>
       <c r="S42" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="T42">
         <v>9</v>
@@ -3527,24 +3515,24 @@
         <v>28</v>
       </c>
       <c r="AA42" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B43" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C43" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D43" t="s">
         <v>28</v>
       </c>
       <c r="E43" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F43" t="s">
         <v>30</v>
@@ -3553,13 +3541,13 @@
         <v>31</v>
       </c>
       <c r="H43" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I43" t="s">
         <v>32</v>
       </c>
       <c r="J43" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L43" t="s">
         <v>43</v>
@@ -3577,7 +3565,7 @@
         <v>0</v>
       </c>
       <c r="S43" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="T43">
         <v>9</v>
@@ -3586,18 +3574,18 @@
         <v>28</v>
       </c>
       <c r="AA43" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B44" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C44" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D44" t="s">
         <v>28</v>
@@ -3612,13 +3600,13 @@
         <v>31</v>
       </c>
       <c r="H44" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I44" t="s">
         <v>32</v>
       </c>
       <c r="J44" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L44" t="s">
         <v>43</v>
@@ -3636,7 +3624,7 @@
         <v>0</v>
       </c>
       <c r="S44" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="T44">
         <v>9</v>
@@ -3645,24 +3633,24 @@
         <v>28</v>
       </c>
       <c r="AA44" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B45" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C45" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D45" t="s">
         <v>28</v>
       </c>
       <c r="E45" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F45" t="s">
         <v>30</v>
@@ -3671,13 +3659,13 @@
         <v>31</v>
       </c>
       <c r="H45" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I45" t="s">
         <v>32</v>
       </c>
       <c r="J45" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L45" t="s">
         <v>43</v>
@@ -3695,7 +3683,7 @@
         <v>0</v>
       </c>
       <c r="S45" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="T45">
         <v>9</v>
@@ -3704,18 +3692,18 @@
         <v>28</v>
       </c>
       <c r="AA45" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B46" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C46" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D46" t="s">
         <v>28</v>
@@ -3730,13 +3718,13 @@
         <v>31</v>
       </c>
       <c r="H46" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I46" t="s">
         <v>32</v>
       </c>
       <c r="J46" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L46" t="s">
         <v>43</v>
@@ -3754,7 +3742,7 @@
         <v>0</v>
       </c>
       <c r="S46" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="T46">
         <v>9</v>
@@ -3763,18 +3751,18 @@
         <v>28</v>
       </c>
       <c r="AA46" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>97</v>
+      </c>
+      <c r="B47" t="s">
         <v>100</v>
       </c>
-      <c r="B47" t="s">
-        <v>103</v>
-      </c>
       <c r="C47" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D47" t="s">
         <v>28</v>
@@ -3789,13 +3777,13 @@
         <v>31</v>
       </c>
       <c r="H47" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I47" t="s">
         <v>32</v>
       </c>
       <c r="J47" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L47" t="s">
         <v>43</v>
@@ -3813,7 +3801,7 @@
         <v>0</v>
       </c>
       <c r="S47" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="T47">
         <v>9</v>
@@ -3822,18 +3810,18 @@
         <v>28</v>
       </c>
       <c r="AA47" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="48" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B48" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C48" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D48" t="s">
         <v>28</v>
@@ -3848,13 +3836,13 @@
         <v>31</v>
       </c>
       <c r="H48" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="I48" t="s">
         <v>32</v>
       </c>
       <c r="J48" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="L48" t="s">
         <v>33</v>
@@ -3872,7 +3860,7 @@
         <v>0</v>
       </c>
       <c r="S48" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="T48">
         <v>9</v>
@@ -3881,18 +3869,18 @@
         <v>28</v>
       </c>
       <c r="AA48" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="49" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B49" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C49" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D49" t="s">
         <v>28</v>
@@ -3907,13 +3895,13 @@
         <v>31</v>
       </c>
       <c r="H49" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="I49" t="s">
         <v>32</v>
       </c>
       <c r="J49" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="L49" t="s">
         <v>43</v>
@@ -3931,7 +3919,7 @@
         <v>0</v>
       </c>
       <c r="S49" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="T49">
         <v>9</v>
@@ -3940,24 +3928,24 @@
         <v>28</v>
       </c>
       <c r="AA49" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="50" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B50" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C50" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D50" t="s">
         <v>28</v>
       </c>
       <c r="E50" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F50" t="s">
         <v>30</v>
@@ -3966,13 +3954,13 @@
         <v>31</v>
       </c>
       <c r="H50" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I50" t="s">
         <v>32</v>
       </c>
       <c r="J50" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L50" t="s">
         <v>43</v>
@@ -3990,7 +3978,7 @@
         <v>0</v>
       </c>
       <c r="S50" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="T50">
         <v>9</v>
@@ -3999,18 +3987,18 @@
         <v>28</v>
       </c>
       <c r="AA50" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="51" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B51" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C51" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D51" t="s">
         <v>28</v>
@@ -4025,13 +4013,13 @@
         <v>31</v>
       </c>
       <c r="H51" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I51" t="s">
         <v>32</v>
       </c>
       <c r="J51" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="L51" t="s">
         <v>43</v>
@@ -4049,7 +4037,7 @@
         <v>0</v>
       </c>
       <c r="S51" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="T51">
         <v>9</v>
@@ -4058,18 +4046,18 @@
         <v>28</v>
       </c>
       <c r="AA51" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="52" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B52" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C52" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D52" t="s">
         <v>28</v>
@@ -4084,13 +4072,13 @@
         <v>31</v>
       </c>
       <c r="H52" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="I52" t="s">
         <v>32</v>
       </c>
       <c r="J52" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="L52" t="s">
         <v>43</v>
@@ -4108,7 +4096,7 @@
         <v>0</v>
       </c>
       <c r="S52" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T52">
         <v>9</v>
@@ -4117,24 +4105,24 @@
         <v>28</v>
       </c>
       <c r="AA52" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="53" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B53" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C53" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D53" t="s">
         <v>28</v>
       </c>
       <c r="E53" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F53" t="s">
         <v>30</v>
@@ -4143,13 +4131,13 @@
         <v>31</v>
       </c>
       <c r="H53" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I53" t="s">
         <v>32</v>
       </c>
       <c r="J53" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="L53" t="s">
         <v>43</v>
@@ -4167,7 +4155,7 @@
         <v>0</v>
       </c>
       <c r="S53" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="T53">
         <v>9</v>
@@ -4176,24 +4164,24 @@
         <v>28</v>
       </c>
       <c r="AA53" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="54" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B54" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C54" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D54" t="s">
         <v>28</v>
       </c>
       <c r="E54" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F54" t="s">
         <v>30</v>
@@ -4226,7 +4214,7 @@
         <v>0</v>
       </c>
       <c r="S54" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="T54">
         <v>9</v>
@@ -4235,18 +4223,18 @@
         <v>28</v>
       </c>
       <c r="AA54" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="55" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B55" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C55" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D55" t="s">
         <v>28</v>
@@ -4285,7 +4273,7 @@
         <v>0</v>
       </c>
       <c r="S55" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="T55">
         <v>9</v>
@@ -4294,18 +4282,18 @@
         <v>28</v>
       </c>
       <c r="AA55" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="56" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B56" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C56" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D56" t="s">
         <v>28</v>
@@ -4344,7 +4332,7 @@
         <v>0</v>
       </c>
       <c r="S56" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="T56">
         <v>9</v>
@@ -4353,18 +4341,18 @@
         <v>28</v>
       </c>
       <c r="AA56" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="57" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B57" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C57" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D57" t="s">
         <v>28</v>
@@ -4379,13 +4367,13 @@
         <v>31</v>
       </c>
       <c r="H57" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="I57" t="s">
         <v>32</v>
       </c>
       <c r="J57" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="L57" t="s">
         <v>43</v>
@@ -4403,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="S57" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="T57">
         <v>9</v>
@@ -4412,18 +4400,18 @@
         <v>28</v>
       </c>
       <c r="AA57" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="58" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B58" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C58" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D58" t="s">
         <v>28</v>
@@ -4438,13 +4426,13 @@
         <v>31</v>
       </c>
       <c r="H58" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I58" t="s">
         <v>32</v>
       </c>
       <c r="J58" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="L58" t="s">
         <v>43</v>
@@ -4462,7 +4450,7 @@
         <v>0</v>
       </c>
       <c r="S58" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="T58">
         <v>9</v>
@@ -4471,18 +4459,18 @@
         <v>28</v>
       </c>
       <c r="AA58" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="59" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B59" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C59" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D59" t="s">
         <v>28</v>
@@ -4521,7 +4509,7 @@
         <v>0</v>
       </c>
       <c r="S59" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="T59">
         <v>9</v>
@@ -4530,18 +4518,18 @@
         <v>28</v>
       </c>
       <c r="AA59" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B60" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C60" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D60" t="s">
         <v>28</v>
@@ -4556,13 +4544,13 @@
         <v>31</v>
       </c>
       <c r="H60" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I60" t="s">
         <v>32</v>
       </c>
       <c r="J60" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L60" t="s">
         <v>43</v>
@@ -4580,7 +4568,7 @@
         <v>0</v>
       </c>
       <c r="S60" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="T60">
         <v>2</v>
@@ -4589,18 +4577,18 @@
         <v>28</v>
       </c>
       <c r="AA60" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="61" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B61" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C61" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D61" t="s">
         <v>28</v>
@@ -4615,13 +4603,13 @@
         <v>31</v>
       </c>
       <c r="H61" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="I61" t="s">
         <v>32</v>
       </c>
       <c r="J61" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="L61" t="s">
         <v>43</v>
@@ -4639,7 +4627,7 @@
         <v>0</v>
       </c>
       <c r="S61" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="T61">
         <v>9</v>
@@ -4648,18 +4636,18 @@
         <v>28</v>
       </c>
       <c r="AA61" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="62" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B62" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C62" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D62" t="s">
         <v>28</v>
@@ -4674,13 +4662,13 @@
         <v>31</v>
       </c>
       <c r="H62" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I62" t="s">
         <v>32</v>
       </c>
       <c r="J62" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L62" t="s">
         <v>43</v>
@@ -4698,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="S62" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="T62">
         <v>9</v>
@@ -4707,39 +4695,39 @@
         <v>28</v>
       </c>
       <c r="AA62" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B63" t="s">
+        <v>179</v>
+      </c>
+      <c r="C63" t="s">
+        <v>179</v>
+      </c>
+      <c r="D63" t="s">
+        <v>28</v>
+      </c>
+      <c r="E63" t="s">
+        <v>113</v>
+      </c>
+      <c r="F63" t="s">
+        <v>30</v>
+      </c>
+      <c r="G63" t="s">
+        <v>31</v>
+      </c>
+      <c r="H63" t="s">
         <v>183</v>
       </c>
-      <c r="C63" t="s">
+      <c r="I63" t="s">
+        <v>32</v>
+      </c>
+      <c r="J63" t="s">
         <v>183</v>
-      </c>
-      <c r="D63" t="s">
-        <v>28</v>
-      </c>
-      <c r="E63" t="s">
-        <v>116</v>
-      </c>
-      <c r="F63" t="s">
-        <v>30</v>
-      </c>
-      <c r="G63" t="s">
-        <v>31</v>
-      </c>
-      <c r="H63" t="s">
-        <v>187</v>
-      </c>
-      <c r="I63" t="s">
-        <v>32</v>
-      </c>
-      <c r="J63" t="s">
-        <v>187</v>
       </c>
       <c r="L63" t="s">
         <v>43</v>
@@ -4757,7 +4745,7 @@
         <v>0</v>
       </c>
       <c r="S63" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="T63">
         <v>9</v>
@@ -4766,18 +4754,18 @@
         <v>28</v>
       </c>
       <c r="AA63" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="64" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B64" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C64" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D64" t="s">
         <v>28</v>
@@ -4792,13 +4780,13 @@
         <v>31</v>
       </c>
       <c r="H64" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I64" t="s">
         <v>32</v>
       </c>
       <c r="J64" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L64" t="s">
         <v>43</v>
@@ -4816,7 +4804,7 @@
         <v>0</v>
       </c>
       <c r="S64" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="T64">
         <v>9</v>
@@ -4825,24 +4813,24 @@
         <v>28</v>
       </c>
       <c r="AA64" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="65" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B65" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C65" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D65" t="s">
         <v>28</v>
       </c>
       <c r="E65" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F65" t="s">
         <v>30</v>
@@ -4851,13 +4839,13 @@
         <v>31</v>
       </c>
       <c r="H65" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I65" t="s">
         <v>32</v>
       </c>
       <c r="J65" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L65" t="s">
         <v>43</v>
@@ -4875,7 +4863,7 @@
         <v>0</v>
       </c>
       <c r="S65" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="T65">
         <v>9</v>
@@ -4884,39 +4872,39 @@
         <v>28</v>
       </c>
       <c r="AA65" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="66" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>179</v>
+      </c>
+      <c r="B66" t="s">
+        <v>126</v>
+      </c>
+      <c r="C66" t="s">
+        <v>179</v>
+      </c>
+      <c r="D66" t="s">
+        <v>28</v>
+      </c>
+      <c r="E66" t="s">
+        <v>132</v>
+      </c>
+      <c r="F66" t="s">
+        <v>30</v>
+      </c>
+      <c r="G66" t="s">
+        <v>31</v>
+      </c>
+      <c r="H66" t="s">
         <v>183</v>
       </c>
-      <c r="B66" t="s">
-        <v>129</v>
-      </c>
-      <c r="C66" t="s">
+      <c r="I66" t="s">
+        <v>32</v>
+      </c>
+      <c r="J66" t="s">
         <v>183</v>
-      </c>
-      <c r="D66" t="s">
-        <v>28</v>
-      </c>
-      <c r="E66" t="s">
-        <v>135</v>
-      </c>
-      <c r="F66" t="s">
-        <v>30</v>
-      </c>
-      <c r="G66" t="s">
-        <v>31</v>
-      </c>
-      <c r="H66" t="s">
-        <v>187</v>
-      </c>
-      <c r="I66" t="s">
-        <v>32</v>
-      </c>
-      <c r="J66" t="s">
-        <v>187</v>
       </c>
       <c r="L66" t="s">
         <v>43</v>
@@ -4934,7 +4922,7 @@
         <v>0</v>
       </c>
       <c r="S66" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="T66">
         <v>9</v>
@@ -4943,18 +4931,18 @@
         <v>28</v>
       </c>
       <c r="AA66" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="67" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B67" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C67" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D67" t="s">
         <v>28</v>
@@ -4969,13 +4957,13 @@
         <v>31</v>
       </c>
       <c r="H67" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I67" t="s">
         <v>32</v>
       </c>
       <c r="J67" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L67" t="s">
         <v>43</v>
@@ -4993,7 +4981,7 @@
         <v>0</v>
       </c>
       <c r="S67" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="T67">
         <v>9</v>
@@ -5002,24 +4990,24 @@
         <v>28</v>
       </c>
       <c r="AA67" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="68" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B68" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C68" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D68" t="s">
         <v>28</v>
       </c>
       <c r="E68" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F68" t="s">
         <v>30</v>
@@ -5028,13 +5016,13 @@
         <v>31</v>
       </c>
       <c r="H68" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I68" t="s">
         <v>32</v>
       </c>
       <c r="J68" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L68" t="s">
         <v>43</v>
@@ -5052,7 +5040,7 @@
         <v>0</v>
       </c>
       <c r="S68" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="T68">
         <v>9</v>
@@ -5061,18 +5049,18 @@
         <v>28</v>
       </c>
       <c r="AA68" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="69" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B69" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C69" t="s">
-        <v>184</v>
+        <v>136</v>
       </c>
       <c r="D69" t="s">
         <v>28</v>
@@ -5087,13 +5075,13 @@
         <v>31</v>
       </c>
       <c r="H69" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I69" t="s">
         <v>32</v>
       </c>
       <c r="J69" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L69" t="s">
         <v>43</v>
@@ -5111,7 +5099,7 @@
         <v>0</v>
       </c>
       <c r="S69" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="T69">
         <v>9</v>
@@ -5120,18 +5108,18 @@
         <v>28</v>
       </c>
       <c r="AA69" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="70" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>136</v>
+      </c>
+      <c r="B70" t="s">
         <v>139</v>
       </c>
-      <c r="B70" t="s">
-        <v>143</v>
-      </c>
       <c r="C70" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D70" t="s">
         <v>28</v>
@@ -5146,13 +5134,13 @@
         <v>31</v>
       </c>
       <c r="H70" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I70" t="s">
         <v>32</v>
       </c>
       <c r="J70" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L70" t="s">
         <v>43</v>
@@ -5170,7 +5158,7 @@
         <v>0</v>
       </c>
       <c r="S70" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="T70">
         <v>9</v>
@@ -5179,18 +5167,18 @@
         <v>28</v>
       </c>
       <c r="AA70" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="71" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B71" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C71" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D71" t="s">
         <v>28</v>
@@ -5205,13 +5193,13 @@
         <v>31</v>
       </c>
       <c r="H71" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I71" t="s">
         <v>32</v>
       </c>
       <c r="J71" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="L71" t="s">
         <v>33</v>
@@ -5229,7 +5217,7 @@
         <v>0</v>
       </c>
       <c r="S71" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="T71">
         <v>9</v>
@@ -5238,18 +5226,18 @@
         <v>28</v>
       </c>
       <c r="AA71" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="72" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B72" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C72" t="s">
-        <v>184</v>
+        <v>136</v>
       </c>
       <c r="D72" t="s">
         <v>28</v>
@@ -5264,13 +5252,13 @@
         <v>31</v>
       </c>
       <c r="H72" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="I72" t="s">
         <v>32</v>
       </c>
       <c r="J72" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="L72" t="s">
         <v>43</v>
@@ -5288,7 +5276,7 @@
         <v>0</v>
       </c>
       <c r="S72" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="T72">
         <v>9</v>
@@ -5297,24 +5285,24 @@
         <v>28</v>
       </c>
       <c r="AA72" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="73" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B73" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C73" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D73" t="s">
         <v>28</v>
       </c>
       <c r="E73" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F73" t="s">
         <v>30</v>
@@ -5323,13 +5311,13 @@
         <v>31</v>
       </c>
       <c r="H73" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="I73" t="s">
         <v>32</v>
       </c>
       <c r="J73" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="L73" t="s">
         <v>43</v>
@@ -5347,7 +5335,7 @@
         <v>0</v>
       </c>
       <c r="S73" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="T73">
         <v>9</v>
@@ -5356,18 +5344,18 @@
         <v>28</v>
       </c>
       <c r="AA73" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="74" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B74" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C74" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D74" t="s">
         <v>28</v>
@@ -5382,13 +5370,13 @@
         <v>31</v>
       </c>
       <c r="H74" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="I74" t="s">
         <v>32</v>
       </c>
       <c r="J74" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="L74" t="s">
         <v>43</v>
@@ -5406,7 +5394,7 @@
         <v>0</v>
       </c>
       <c r="S74" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="T74">
         <v>9</v>
@@ -5415,18 +5403,18 @@
         <v>28</v>
       </c>
       <c r="AA74" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="75" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B75" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" t="s">
         <v>139</v>
-      </c>
-      <c r="C75" t="s">
-        <v>143</v>
       </c>
       <c r="D75" t="s">
         <v>28</v>
@@ -5441,13 +5429,13 @@
         <v>31</v>
       </c>
       <c r="H75" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I75" t="s">
         <v>32</v>
       </c>
       <c r="J75" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="L75" t="s">
         <v>43</v>
@@ -5465,7 +5453,7 @@
         <v>0</v>
       </c>
       <c r="S75" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="T75">
         <v>9</v>
@@ -5474,18 +5462,18 @@
         <v>28</v>
       </c>
       <c r="AA75" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="76" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B76" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C76" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D76" t="s">
         <v>28</v>
@@ -5500,13 +5488,13 @@
         <v>31</v>
       </c>
       <c r="H76" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I76" t="s">
         <v>32</v>
       </c>
       <c r="J76" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L76" t="s">
         <v>43</v>
@@ -5524,7 +5512,7 @@
         <v>0</v>
       </c>
       <c r="S76" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="T76">
         <v>8</v>
@@ -5533,18 +5521,18 @@
         <v>28</v>
       </c>
       <c r="AA76" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="77" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B77" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C77" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D77" t="s">
         <v>28</v>
@@ -5559,13 +5547,13 @@
         <v>31</v>
       </c>
       <c r="H77" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I77" t="s">
         <v>32</v>
       </c>
       <c r="J77" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="L77" t="s">
         <v>43</v>
@@ -5583,7 +5571,7 @@
         <v>0</v>
       </c>
       <c r="S77" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="T77">
         <v>9</v>
@@ -5592,18 +5580,18 @@
         <v>28</v>
       </c>
       <c r="AA77" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="78" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B78" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C78" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D78" t="s">
         <v>28</v>
@@ -5618,13 +5606,13 @@
         <v>31</v>
       </c>
       <c r="H78" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I78" t="s">
         <v>32</v>
       </c>
       <c r="J78" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="L78" t="s">
         <v>33</v>
@@ -5642,7 +5630,7 @@
         <v>0</v>
       </c>
       <c r="S78" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="T78">
         <v>9</v>
@@ -5651,7 +5639,7 @@
         <v>28</v>
       </c>
       <c r="AA78" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -5671,10 +5659,10 @@
         <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -5704,7 +5692,7 @@
         <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -5726,7 +5714,7 @@
         <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -5748,7 +5736,7 @@
         <v>60</v>
       </c>
       <c r="B8" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C8">
         <v>4</v>
@@ -5770,7 +5758,7 @@
         <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -5800,7 +5788,7 @@
         <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C13">
         <v>4</v>
@@ -5808,10 +5796,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -5819,10 +5807,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C15">
         <v>4</v>
@@ -5830,10 +5818,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C16">
         <v>5</v>
@@ -5841,18 +5829,18 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B17" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B18" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C18">
         <v>4</v>
@@ -5860,10 +5848,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B19" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -5871,10 +5859,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B20" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C20">
         <v>2</v>
@@ -5882,26 +5870,26 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B21" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B22" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B23" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C23">
         <v>4</v>
@@ -5909,10 +5897,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B24" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C24">
         <v>3</v>
@@ -5920,10 +5908,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B25" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C25">
         <v>3</v>
@@ -5931,10 +5919,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B26" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C26">
         <v>5</v>
@@ -5942,10 +5930,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -5953,10 +5941,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B28" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C28">
         <v>4</v>
@@ -5964,18 +5952,18 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>123</v>
+      </c>
+      <c r="B29" t="s">
         <v>126</v>
-      </c>
-      <c r="B29" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B30" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C30">
         <v>3</v>
@@ -5983,10 +5971,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B31" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C31">
         <v>4</v>
@@ -5994,10 +5982,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B32" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -6005,10 +5993,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B33" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C33">
         <v>2</v>
@@ -6023,6 +6011,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="27" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" customWidth="1"/>
+    <col min="4" max="4" width="35.5703125" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
@@ -6035,10 +6029,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>32</v>
@@ -6055,73 +6049,73 @@
         <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E2" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="F2" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>162</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>169</v>
       </c>
       <c r="D3" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
-        <v>88</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>162</v>
       </c>
       <c r="D4" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E4" t="s">
-        <v>94</v>
+        <v>162</v>
       </c>
       <c r="F4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="C5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E5" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F5" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>